<commit_message>
Phase 1 UX Grid Editor and push last changes
</commit_message>
<xml_diff>
--- a/docs/Design/Grimrock Items.xlsx
+++ b/docs/Design/Grimrock Items.xlsx
@@ -5,15 +5,16 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Development\GrimrockPrototype\docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Development\GrimrockPrototype\docs\Design\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3116F8E0-FE5F-4F15-85B2-43038CB04689}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D9F7887-DB5F-4A3E-8F46-D80EA39499DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9330" yWindow="6855" windowWidth="40710" windowHeight="23520" xr2:uid="{9BA64EF4-07C9-4015-A37D-185E14582EAA}"/>
+    <workbookView xWindow="17100" yWindow="5250" windowWidth="28365" windowHeight="23520" activeTab="1" xr2:uid="{9BA64EF4-07C9-4015-A37D-185E14582EAA}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
+    <sheet name="Feuil2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="260" uniqueCount="126">
   <si>
     <t>Bouton</t>
   </si>
@@ -190,19 +191,527 @@
   </si>
   <si>
     <t>Torche</t>
+  </si>
+  <si>
+    <t>Objet</t>
+  </si>
+  <si>
+    <t>Catégorie</t>
+  </si>
+  <si>
+    <t>Classe / base</t>
+  </si>
+  <si>
+    <t>Événements émis</t>
+  </si>
+  <si>
+    <t>État initial</t>
+  </si>
+  <si>
+    <t>Mechanism</t>
+  </si>
+  <si>
+    <t>AGridButtonActor</t>
+  </si>
+  <si>
+    <t>OnActivate</t>
+  </si>
+  <si>
+    <t>relâché / pressé</t>
+  </si>
+  <si>
+    <t>clic / Use</t>
+  </si>
+  <si>
+    <t>Bouton mural</t>
+  </si>
+  <si>
+    <t>AGridLeverActor</t>
+  </si>
+  <si>
+    <r>
+      <t>OnActivate</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>OnDeactivate</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>OnToggle</t>
+    </r>
+  </si>
+  <si>
+    <t>activé / désactivé</t>
+  </si>
+  <si>
+    <t>AGridPressurePlateActor</t>
+  </si>
+  <si>
+    <t>désactivée par défaut</t>
+  </si>
+  <si>
+    <t>marcher dessus / item</t>
+  </si>
+  <si>
+    <t>Trigger</t>
+  </si>
+  <si>
+    <t>AGridTriggerActor</t>
+  </si>
+  <si>
+    <r>
+      <t>OnEnter</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>OnExit</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>OnActivate</t>
+    </r>
+  </si>
+  <si>
+    <t>actif / inactif</t>
+  </si>
+  <si>
+    <t>marcher dessus</t>
+  </si>
+  <si>
+    <t>Receptacle</t>
+  </si>
+  <si>
+    <r>
+      <t>AGridReceptacleActor</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> ou </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>AGridLockActor</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>OnInsertItem</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>OnUnlock</t>
+    </r>
+  </si>
+  <si>
+    <t>verrouillée</t>
+  </si>
+  <si>
+    <t>ajout clé</t>
+  </si>
+  <si>
+    <r>
+      <t>Mechanism</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> / </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>Decoration</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> / </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>Light</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">acteur générique ou futur </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>AGridRuneActor</t>
+    </r>
+  </si>
+  <si>
+    <t>activée / désactivée</t>
+  </si>
+  <si>
+    <t>clic / marche / lien</t>
+  </si>
+  <si>
+    <t>AGridTimerActor</t>
+  </si>
+  <si>
+    <t>OnTimer</t>
+  </si>
+  <si>
+    <t>arrêté</t>
+  </si>
+  <si>
+    <t>script / lien</t>
+  </si>
+  <si>
+    <t>AGridReceptacleActor</t>
+  </si>
+  <si>
+    <r>
+      <t>OnInsertItem</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>OnRemoveItem</t>
+    </r>
+  </si>
+  <si>
+    <t>vide / occupée</t>
+  </si>
+  <si>
+    <t>ajout / retrait item</t>
+  </si>
+  <si>
+    <t>vide / occupé</t>
+  </si>
+  <si>
+    <t>ajout / retrait torche</t>
+  </si>
+  <si>
+    <t>Autel</t>
+  </si>
+  <si>
+    <t>Bol d’offrande</t>
+  </si>
+  <si>
+    <t>OnInsertItem</t>
+  </si>
+  <si>
+    <t>vide</t>
+  </si>
+  <si>
+    <t>ajout pièce</t>
+  </si>
+  <si>
+    <t>AGridDoorActor</t>
+  </si>
+  <si>
+    <t>optionnel</t>
+  </si>
+  <si>
+    <t>ouverte / fermée / verrouillée</t>
+  </si>
+  <si>
+    <t>mécanisme / lien</t>
+  </si>
+  <si>
+    <t>Porte secrète</t>
+  </si>
+  <si>
+    <t>AGridSecretDoorActor</t>
+  </si>
+  <si>
+    <t>ouverte / fermée / cachée</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">futur </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>AGridTrapdoorActor</t>
+    </r>
+  </si>
+  <si>
+    <t>ouverte / fermée</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">futur </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>AGridTeleporterActor</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>OnEnter</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> optionnel</t>
+    </r>
+  </si>
+  <si>
+    <t>marche dessus / lien</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">futur </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>AGridItemActor</t>
+    </r>
+  </si>
+  <si>
+    <t>aucun</t>
+  </si>
+  <si>
+    <t>inventaire / serrure</t>
+  </si>
+  <si>
+    <t>inventaire / fente</t>
+  </si>
+  <si>
+    <r>
+      <t>Item</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> ou </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>Light</t>
+    </r>
+  </si>
+  <si>
+    <t>aucun ou optionnel</t>
+  </si>
+  <si>
+    <t>allumée / éteinte</t>
+  </si>
+  <si>
+    <t>inventaire / support</t>
+  </si>
+  <si>
+    <t>WallInscription</t>
+  </si>
+  <si>
+    <t>Readable</t>
+  </si>
+  <si>
+    <t>classe existante WallInscription</t>
+  </si>
+  <si>
+    <t>OnUse</t>
+  </si>
+  <si>
+    <t>touche F / Use</t>
+  </si>
+  <si>
+    <t>Spawn joueur</t>
+  </si>
+  <si>
+    <t>Spawn</t>
+  </si>
+  <si>
+    <t>marker / données de niveau</t>
+  </si>
+  <si>
+    <t>runtime init</t>
+  </si>
+  <si>
+    <t>Spawn monstre</t>
+  </si>
+  <si>
+    <t>futur spawn actor / données</t>
+  </si>
+  <si>
+    <r>
+      <t>OnSpawn</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> optionnel</t>
+    </r>
+  </si>
+  <si>
+    <t>lien / script</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial Unicode MS"/>
     </font>
   </fonts>
   <fills count="2">
@@ -225,10 +734,19 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -951,4 +1469,522 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3D2E4C8A-2B67-4FE8-8DB1-70437B650494}">
+  <dimension ref="A1:F25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25"/>
+  <cols>
+    <col min="1" max="1" width="16.75" customWidth="1"/>
+    <col min="2" max="2" width="16.25" customWidth="1"/>
+    <col min="3" max="3" width="22.125" customWidth="1"/>
+    <col min="4" max="4" width="23.625" customWidth="1"/>
+    <col min="5" max="5" width="26.75" customWidth="1"/>
+    <col min="6" max="6" width="26.625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" ht="15">
+      <c r="A1" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
+      <c r="A2" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6">
+      <c r="A3" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6">
+      <c r="A4" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="27">
+      <c r="A5" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="27">
+      <c r="A6" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6">
+      <c r="A7" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="27">
+      <c r="A8" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="28.5">
+      <c r="A9" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6">
+      <c r="A10" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6">
+      <c r="A11" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6">
+      <c r="A12" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6">
+      <c r="A13" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="F13" s="3" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6">
+      <c r="A14" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="F14" s="3" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6">
+      <c r="A15" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="F15" s="3" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6">
+      <c r="A16" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="E16" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="F16" s="3" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6">
+      <c r="A17" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="F17" s="3" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6">
+      <c r="A18" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="D18" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="E18" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="F18" s="3" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6">
+      <c r="A19" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="D19" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="E19" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="F19" s="3" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6">
+      <c r="A20" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="D20" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="E20" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="F20" s="3" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6">
+      <c r="A21" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="C21" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="D21" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="E21" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="F21" s="3" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6">
+      <c r="A22" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="D22" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="E22" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="F22" s="3" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" ht="28.5">
+      <c r="A23" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="D23" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="E23" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="F23" s="3" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" ht="28.5">
+      <c r="A24" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="B24" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="D24" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="E24" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="F24" s="3" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" ht="28.5">
+      <c r="A25" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="C25" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="D25" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="E25" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="F25" s="3" t="s">
+        <v>125</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>